<commit_message>
UX-Polish: Legende-Farben, Borders, Spaltenbreiten
- Legende: Font-Bug gefixt - GT/NST/Fobi hatten schwarzen
  Hintergrund statt keinen (fn.color.rgb Zugriff auf None).
  Jetzt sauberer _leg_font() Helper der Color-Objekt korrekt
  weitergibt.
- Besetzungs-Zeile: border=THIN auf Namenszelle (war borderlos)
- Spaltenbreite: min 4.0 statt 3.8 (besser lesbar bei 31 Tagen)

Verifiziert:
- Alle 31 XML-Dateien parsebar
- 5 dxf-Styles mit jeweils font+fill (kein Crash)
- DV: 12 Ranges, 120 chars (kein overflow)
- 0 merge overlaps in allen 16 Sheets
- Legende: GT/NST/Fobi = rot font, kein fill (korrekt)
- Alle 12 Monate: fitToPage, landscape, freeze=B6

https://claude.ai/code/session_01QQEWdtZ1agPkU2NjoafpqQ
</commit_message>
<xml_diff>
--- a/Dienstplan_2026_neu.xlsx
+++ b/Dienstplan_2026_neu.xlsx
@@ -513,7 +513,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -16941,36 +16941,36 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19249,37 +19249,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
-    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21617,36 +21617,36 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -23916,37 +23916,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
-    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -35413,37 +35413,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
-    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -37713,34 +37713,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -39827,37 +39827,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
-    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -42112,36 +42112,36 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -44345,37 +44345,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
-    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -46697,36 +46697,36 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -49002,37 +49002,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
-    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -51357,37 +51357,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="3.8" customWidth="1" min="2" max="2"/>
-    <col width="3.8" customWidth="1" min="3" max="3"/>
-    <col width="3.8" customWidth="1" min="4" max="4"/>
-    <col width="3.8" customWidth="1" min="5" max="5"/>
-    <col width="3.8" customWidth="1" min="6" max="6"/>
-    <col width="3.8" customWidth="1" min="7" max="7"/>
-    <col width="3.8" customWidth="1" min="8" max="8"/>
-    <col width="3.8" customWidth="1" min="9" max="9"/>
-    <col width="3.8" customWidth="1" min="10" max="10"/>
-    <col width="3.8" customWidth="1" min="11" max="11"/>
-    <col width="3.8" customWidth="1" min="12" max="12"/>
-    <col width="3.8" customWidth="1" min="13" max="13"/>
-    <col width="3.8" customWidth="1" min="14" max="14"/>
-    <col width="3.8" customWidth="1" min="15" max="15"/>
-    <col width="3.8" customWidth="1" min="16" max="16"/>
-    <col width="3.8" customWidth="1" min="17" max="17"/>
-    <col width="3.8" customWidth="1" min="18" max="18"/>
-    <col width="3.8" customWidth="1" min="19" max="19"/>
-    <col width="3.8" customWidth="1" min="20" max="20"/>
-    <col width="3.8" customWidth="1" min="21" max="21"/>
-    <col width="3.8" customWidth="1" min="22" max="22"/>
-    <col width="3.8" customWidth="1" min="23" max="23"/>
-    <col width="3.8" customWidth="1" min="24" max="24"/>
-    <col width="3.8" customWidth="1" min="25" max="25"/>
-    <col width="3.8" customWidth="1" min="26" max="26"/>
-    <col width="3.8" customWidth="1" min="27" max="27"/>
-    <col width="3.8" customWidth="1" min="28" max="28"/>
-    <col width="3.8" customWidth="1" min="29" max="29"/>
-    <col width="3.8" customWidth="1" min="30" max="30"/>
-    <col width="3.8" customWidth="1" min="31" max="31"/>
-    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>